<commit_message>
Exercise 2.A Normalization Practice for Week-02
</commit_message>
<xml_diff>
--- a/week-02/Ex2A_events_normalized.xlsx
+++ b/week-02/Ex2A_events_normalized.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/04a19e4a9bb9275a/Desktop/DataAnalytics/week-02/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="33" documentId="8_{FD532578-2C22-41AD-8277-93B8A0AC55B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1944A7F6-607B-4CA0-8393-9D056A9886BC}"/>
+  <xr:revisionPtr revIDLastSave="111" documentId="8_{FD532578-2C22-41AD-8277-93B8A0AC55B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9B499273-8BC5-4BA9-B7FE-BD45570322D2}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="14676" windowHeight="13056" xr2:uid="{5091876E-AF08-41C4-B976-D2AB9D8B455C}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="12780" windowHeight="13056" xr2:uid="{5091876E-AF08-41C4-B976-D2AB9D8B455C}"/>
   </bookViews>
   <sheets>
     <sheet name="events_sample" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="141">
   <si>
     <t>Event ID</t>
   </si>
@@ -429,6 +429,112 @@
   </si>
   <si>
     <t>5th Table:</t>
+  </si>
+  <si>
+    <t>Event_Category</t>
+  </si>
+  <si>
+    <t>Employee Name</t>
+  </si>
+  <si>
+    <t>Employee Email</t>
+  </si>
+  <si>
+    <t>Employee_Venue_Assignment</t>
+  </si>
+  <si>
+    <t>Role</t>
+  </si>
+  <si>
+    <t>Manager</t>
+  </si>
+  <si>
+    <t>7th Table:</t>
+  </si>
+  <si>
+    <t>6th table:</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>***Originally my 3rd table (which was Venue_Directory) had Starlight_CA and DtwnCon_IL twice, so had to remove duplicated data.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>***AI (Copilot) said for table Venue_Employee: It is not normalized</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+This table mixes:
+Employee #
+Venue ID
+Event Manager name
+Manager email
+Example:
+“u1023 – Starlight_CA – Sarah Mitchell – sarah.mitchell@eventdoodle.com”
+Issues:
+Employee # already identifies the employee — so storing the manager name and email again is redundant.
+If Sarah Mitchell changes her email, you’d have to update multiple rows.
+This table is trying to represent two concepts at once:
+Who works at a venue
+Who manages an event
+Fix: Split into two tables:
+A. Employee Table
+Employee # (PK)
+Employee Name
+Employee Email
+B. Employee_Venue_Assignment
+Employee # (FK)
+Venue ID (FK)
+Role (e.g., Manager, Staff)
+This removes redundancy and improves clarity.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+At first I thought this made no sense to do because I thought I needed to "make up" employee information for the Employee Table but in reality we are just seperating the Employee's to their position. Ai did mention that by keeping the email and emplpyee id together it creates data redundancy, which we want to avoid in a normalized database. So I ended up breaking up my Venue_Employee table into two different tables. 
+It also stated that I needed to create a speerate table that highlights the Event Category and the Category Code (with category code being the PK). Correcting my previous tables removed a lot of redundancy and irrelevant data on my tables. It also allowed my tables to be easily modified without the need or needing to alter multiple parts of a table (for example by seperating employee and thier position in another table in relation to their employee id). I also moved my tables around (like put the bridging tables between two tables where the info would need to be pulled from). Because earlier I was just copying and pasting everywhere and just removing information from eaach table little by little so it wasn't flowing correctly.</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -953,8 +1059,8 @@
     <xf numFmtId="0" fontId="0" fillId="34" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -1012,6 +1118,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1331,7 +1441,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8FA38BEC-78EC-44DC-83F3-AA711D021920}">
-  <dimension ref="A1:Q93"/>
+  <dimension ref="A1:Q139"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.33203125" style="1" customWidth="1"/>
@@ -1992,1012 +2102,1281 @@
     </row>
     <row r="14" spans="1:17" s="3" customFormat="1" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="15" spans="1:17" ht="15" thickTop="1" x14ac:dyDescent="0.3"/>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
         <v>100</v>
       </c>
-      <c r="B16" s="5" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A17" s="6" t="s">
+      <c r="B17" s="5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A18" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B17" s="6" t="s">
+      <c r="B18" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A19" s="1">
+        <v>102</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19" s="2">
+        <v>46095</v>
+      </c>
+      <c r="D19" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A20" s="1">
+        <v>103</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C20" s="2">
+        <v>46194</v>
+      </c>
+      <c r="D20" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A21" s="1">
+        <v>104</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C21" s="2">
+        <v>46115</v>
+      </c>
+      <c r="D21" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A22" s="1">
+        <v>105</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C22" s="2">
+        <v>46157</v>
+      </c>
+      <c r="D22" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A23" s="1">
+        <v>106</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C23" s="2">
+        <v>46109</v>
+      </c>
+      <c r="D23" s="1">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A24" s="1">
+        <v>107</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24" s="2">
+        <v>46130</v>
+      </c>
+      <c r="D24" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A25" s="1">
+        <v>108</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" s="2">
+        <v>46144</v>
+      </c>
+      <c r="D25" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A26" s="1">
+        <v>109</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C26" s="2">
+        <v>46181</v>
+      </c>
+      <c r="D26" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A27" s="1">
+        <v>110</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C27" s="2">
+        <v>46215</v>
+      </c>
+      <c r="D27" s="1">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A28" s="1">
+        <v>111</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C28" s="2">
+        <v>46102</v>
+      </c>
+      <c r="D28" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A29" s="1">
+        <v>112</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C29" s="2">
+        <v>46137</v>
+      </c>
+      <c r="D29" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D30" s="2"/>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="D31" s="2"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A32" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D32" s="2"/>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A33" s="1">
+        <v>7</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D33" s="2"/>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A34" s="1">
+        <v>7</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D34" s="2"/>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A35" s="1">
+        <v>2</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="D35" s="2"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A36" s="1">
+        <v>3</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D36" s="2"/>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A37" s="1">
+        <v>6</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D37" s="2"/>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A38" s="1">
+        <v>4</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D38" s="2"/>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A39" s="1">
+        <v>5</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D39" s="2"/>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A40" s="1">
+        <v>3</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D40" s="2"/>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A41" s="1">
+        <v>7</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A42" s="1">
+        <v>2</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A43" s="1">
+        <v>1</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="B45" s="5" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A46" s="6" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A18" s="1">
-        <v>102</v>
-      </c>
-      <c r="B18" s="1" t="s">
+      <c r="B46" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="H46" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="I46" s="1" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A47" s="1" t="s">
         <v>116</v>
       </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A19" s="1">
-        <v>103</v>
-      </c>
-      <c r="B19" s="1" t="s">
+      <c r="B47" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F47" s="1">
+        <v>90026</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="H47" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="I47" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A48" s="1" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A20" s="1">
-        <v>104</v>
-      </c>
-      <c r="B20" s="1" t="s">
+      <c r="B48" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="F48" s="1">
+        <v>78741</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="H48" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="I48" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A49" s="1" t="s">
         <v>117</v>
       </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A21" s="1">
-        <v>105</v>
-      </c>
-      <c r="B21" s="1" t="s">
+      <c r="B49" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="F49" s="1">
+        <v>90046</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="H49" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="I49" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A50" s="1" t="s">
         <v>118</v>
       </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A22" s="1">
-        <v>106</v>
-      </c>
-      <c r="B22" s="1" t="s">
+      <c r="B50" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F50" s="1">
+        <v>60616</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="H50" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I50" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A51" s="1" t="s">
         <v>119</v>
       </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A23" s="1">
-        <v>107</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A24" s="1">
-        <v>108</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A25" s="1">
-        <v>109</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A26" s="1">
-        <v>110</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A27" s="1">
-        <v>111</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A28" s="1">
-        <v>112</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="B33" s="5" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="6" t="s">
-        <v>0</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="D34" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>103</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A35" s="1">
-        <v>102</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D35" s="2">
-        <v>46095</v>
-      </c>
-      <c r="E35" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F35" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A36" s="1">
-        <v>103</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D36" s="2">
-        <v>46194</v>
-      </c>
-      <c r="E36" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F36" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A37" s="1">
-        <v>104</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D37" s="2">
-        <v>46115</v>
-      </c>
-      <c r="E37" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F37" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A38" s="1">
-        <v>105</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D38" s="2">
-        <v>46157</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F38" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A39" s="1">
-        <v>106</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C39" s="1" t="s">
+      <c r="B51" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="D39" s="2">
-        <v>46109</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="F39" s="1">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A40" s="1">
-        <v>107</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D40" s="2">
-        <v>46130</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="F40" s="1">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A41" s="1">
-        <v>108</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="C41" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D41" s="2">
-        <v>46144</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="F41" s="1">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A42" s="1">
-        <v>109</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D42" s="2">
-        <v>46181</v>
-      </c>
-      <c r="E42" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="F42" s="1">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43" s="1">
-        <v>110</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D43" s="2">
-        <v>46215</v>
-      </c>
-      <c r="E43" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="F43" s="1">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A44" s="1">
-        <v>111</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="D44" s="2">
-        <v>46102</v>
-      </c>
-      <c r="E44" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="F44" s="1">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A45" s="1">
-        <v>112</v>
-      </c>
-      <c r="B45" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D45" s="2">
-        <v>46137</v>
-      </c>
-      <c r="E45" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="F45" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A50" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="B50" s="5" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A51" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="B51" s="1" t="s">
-        <v>113</v>
-      </c>
       <c r="C51" s="1" t="s">
-        <v>90</v>
+        <v>63</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>91</v>
+        <v>64</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="F51" s="1" t="s">
-        <v>93</v>
+        <v>65</v>
+      </c>
+      <c r="F51" s="1">
+        <v>10011</v>
       </c>
       <c r="G51" s="1" t="s">
-        <v>96</v>
+        <v>66</v>
       </c>
       <c r="H51" s="1" t="s">
-        <v>94</v>
+        <v>67</v>
       </c>
       <c r="I51" s="1" t="s">
-        <v>95</v>
+        <v>68</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>4</v>
+        <v>25</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>42</v>
+        <v>69</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>43</v>
+        <v>70</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>44</v>
+        <v>71</v>
       </c>
       <c r="F52" s="1">
-        <v>90026</v>
+        <v>97214</v>
       </c>
       <c r="G52" s="1" t="s">
-        <v>98</v>
+        <v>72</v>
       </c>
       <c r="H52" s="1" t="s">
-        <v>45</v>
+        <v>73</v>
       </c>
       <c r="I52" s="1" t="s">
-        <v>46</v>
+        <v>74</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>8</v>
+        <v>28</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>47</v>
+        <v>75</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>48</v>
+        <v>76</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>49</v>
+        <v>77</v>
       </c>
       <c r="F53" s="1">
-        <v>78741</v>
+        <v>48226</v>
       </c>
       <c r="G53" s="1" t="s">
-        <v>50</v>
+        <v>78</v>
       </c>
       <c r="H53" s="1" t="s">
-        <v>51</v>
+        <v>79</v>
       </c>
       <c r="I53" s="1" t="s">
-        <v>52</v>
+        <v>80</v>
       </c>
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>11</v>
+        <v>32</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>53</v>
+        <v>81</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>54</v>
+        <v>64</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>44</v>
+        <v>65</v>
       </c>
       <c r="F54" s="1">
-        <v>90046</v>
+        <v>10012</v>
       </c>
       <c r="G54" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="H54" s="1" t="s">
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="I54" s="1" t="s">
-        <v>56</v>
+        <v>83</v>
       </c>
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="F55" s="1">
+        <v>33132</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="I55" s="1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A57" s="4" t="s">
+        <v>129</v>
+      </c>
+      <c r="B57" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A58" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="B58" s="6" t="s">
+        <v>114</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A59" s="1">
+        <v>102</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A60" s="1">
+        <v>103</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A61" s="1">
+        <v>104</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A62" s="1">
+        <v>105</v>
+      </c>
+      <c r="B62" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="B55" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C55" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="E55" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F55" s="1">
-        <v>60616</v>
-      </c>
-      <c r="G55" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="H55" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I55" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A56" s="1" t="s">
+    </row>
+    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A63" s="1">
+        <v>106</v>
+      </c>
+      <c r="B63" s="1" t="s">
         <v>119</v>
       </c>
-      <c r="B56" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="C56" s="1" t="s">
-        <v>63</v>
-      </c>
-      <c r="D56" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E56" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F56" s="1">
-        <v>10011</v>
-      </c>
-      <c r="G56" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="H56" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="I56" s="1" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A57" s="1" t="s">
+    </row>
+    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A64" s="1">
+        <v>107</v>
+      </c>
+      <c r="B64" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="B57" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C57" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D57" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="E57" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="F57" s="1">
-        <v>60616</v>
-      </c>
-      <c r="G57" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="H57" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="I57" s="1" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A58" s="1" t="s">
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A65" s="1">
+        <v>108</v>
+      </c>
+      <c r="B65" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="B58" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C58" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D58" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="E58" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="F58" s="1">
-        <v>97214</v>
-      </c>
-      <c r="G58" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="H58" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="I58" s="1" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A59" s="1" t="s">
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A66" s="1">
+        <v>109</v>
+      </c>
+      <c r="B66" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="B59" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C59" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="D59" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="E59" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="F59" s="1">
-        <v>48226</v>
-      </c>
-      <c r="G59" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="H59" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="I59" s="1" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A60" s="1" t="s">
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A67" s="1">
+        <v>110</v>
+      </c>
+      <c r="B67" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="B60" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C60" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D60" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="E60" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="F60" s="1">
-        <v>90026</v>
-      </c>
-      <c r="G60" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="H60" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="I60" s="1" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A61" s="1" t="s">
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A68" s="1">
+        <v>111</v>
+      </c>
+      <c r="B68" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="B61" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C61" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D61" s="1" t="s">
-        <v>64</v>
-      </c>
-      <c r="E61" s="1" t="s">
-        <v>65</v>
-      </c>
-      <c r="F61" s="1">
-        <v>10012</v>
-      </c>
-      <c r="G61" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="H61" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="I61" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A62" s="1" t="s">
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A69" s="1">
+        <v>112</v>
+      </c>
+      <c r="B69" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="B62" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="C62" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D62" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="E62" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="F62" s="1">
-        <v>33132</v>
-      </c>
-      <c r="G62" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="H62" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="I62" s="1" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A67" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="B67" s="5" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A68" s="6" t="s">
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A71" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B71" s="5" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A72" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="B68" s="6" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A69" s="1" t="s">
+      <c r="B72" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A73" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="B69" s="1">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A70" s="1" t="s">
+      <c r="B73" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A74" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B70" s="1">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A71" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="B71" s="1">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A72" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="B72" s="1">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A73" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="B73" s="1">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A74" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="B74" s="1">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="B74" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B75" s="1">
+      <c r="B75" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A76" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A77" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A78" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A79" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A80" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A81" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A82" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A83" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A85" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="B85" s="5" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A86" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B86" s="6" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A87" s="1" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A76" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="B76" s="1">
+      <c r="B87" s="1">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A88" s="1" t="s">
         <v>109</v>
       </c>
-    </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A77" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="B77" s="1">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A78" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="B78" s="1">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A79" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="B79" s="1">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A81" s="4" t="s">
-        <v>131</v>
-      </c>
-      <c r="B81" s="5" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A82" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="B82" s="7" t="s">
-        <v>114</v>
-      </c>
-      <c r="C82" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="D82" s="1" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A83" s="1" t="s">
-        <v>108</v>
-      </c>
-      <c r="B83" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="C83" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D83" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A84" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="B84" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="C84" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D84" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A85" s="1" t="s">
-        <v>110</v>
-      </c>
-      <c r="B85" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="C85" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D85" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A86" s="1" t="s">
-        <v>109</v>
-      </c>
-      <c r="B86" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="C86" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D86" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A87" s="1" t="s">
-        <v>124</v>
-      </c>
-      <c r="B87" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="C87" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D87" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A88" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="B88" s="1" t="s">
-        <v>118</v>
-      </c>
-      <c r="C88" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D88" s="1" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="B88" s="1">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B89" s="1" t="s">
+      <c r="B89" s="1">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A90" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B90" s="1">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A91" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B91" s="1">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A92" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B92" s="1">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A93" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B93" s="1">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A94" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="B94" s="1">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A95" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B95" s="1">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A96" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B96" s="1">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A97" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B97" s="1">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A99" s="4" t="s">
+        <v>138</v>
+      </c>
+      <c r="B99" s="5" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A100" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A101" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A102" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A103" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A104" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A105" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A106" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A107" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="B107" s="1" t="s">
         <v>120</v>
       </c>
-      <c r="C89" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D89" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A90" s="1" t="s">
+      <c r="C107" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A108" s="1" t="s">
         <v>112</v>
       </c>
-      <c r="B90" s="1" t="s">
+      <c r="B108" s="1" t="s">
         <v>121</v>
       </c>
-      <c r="C90" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D90" s="1" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A91" s="1" t="s">
+      <c r="C108" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A109" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B91" s="1" t="s">
+      <c r="B109" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="C91" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D91" s="1" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A92" s="1" t="s">
+      <c r="C109" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A110" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="B92" s="1" t="s">
+      <c r="B110" s="1" t="s">
         <v>122</v>
       </c>
-      <c r="C92" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D92" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A93" s="1" t="s">
+      <c r="C110" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A111" s="1" t="s">
         <v>124</v>
       </c>
-      <c r="B93" s="1" t="s">
+      <c r="B111" s="1" t="s">
         <v>123</v>
       </c>
-      <c r="C93" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D93" s="1" t="s">
-        <v>39</v>
-      </c>
+      <c r="C111" s="1" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" ht="409.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A114" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="B114" s="7"/>
+      <c r="C114" s="7"/>
+      <c r="D114" s="7"/>
+      <c r="E114" s="7"/>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A115" s="7"/>
+      <c r="B115" s="7"/>
+      <c r="C115" s="7"/>
+      <c r="D115" s="7"/>
+      <c r="E115" s="7"/>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A116" s="7"/>
+      <c r="B116" s="7"/>
+      <c r="C116" s="7"/>
+      <c r="D116" s="7"/>
+      <c r="E116" s="7"/>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A117" s="7"/>
+      <c r="B117" s="7"/>
+      <c r="C117" s="7"/>
+      <c r="D117" s="7"/>
+      <c r="E117" s="7"/>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A118" s="7"/>
+      <c r="B118" s="7"/>
+      <c r="C118" s="7"/>
+      <c r="D118" s="7"/>
+      <c r="E118" s="7"/>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A119" s="7"/>
+      <c r="B119" s="7"/>
+      <c r="C119" s="7"/>
+      <c r="D119" s="7"/>
+      <c r="E119" s="7"/>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A120" s="7"/>
+      <c r="B120" s="7"/>
+      <c r="C120" s="7"/>
+      <c r="D120" s="7"/>
+      <c r="E120" s="7"/>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A121" s="7"/>
+      <c r="B121" s="7"/>
+      <c r="C121" s="7"/>
+      <c r="D121" s="7"/>
+      <c r="E121" s="7"/>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A122" s="7"/>
+      <c r="B122" s="7"/>
+      <c r="C122" s="7"/>
+      <c r="D122" s="7"/>
+      <c r="E122" s="7"/>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A123" s="7"/>
+      <c r="B123" s="7"/>
+      <c r="C123" s="7"/>
+      <c r="D123" s="7"/>
+      <c r="E123" s="7"/>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A124" s="7"/>
+      <c r="B124" s="7"/>
+      <c r="C124" s="7"/>
+      <c r="D124" s="7"/>
+      <c r="E124" s="7"/>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A125" s="7"/>
+      <c r="B125" s="7"/>
+      <c r="C125" s="7"/>
+      <c r="D125" s="7"/>
+      <c r="E125" s="7"/>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A126" s="7"/>
+      <c r="B126" s="7"/>
+      <c r="C126" s="7"/>
+      <c r="D126" s="7"/>
+      <c r="E126" s="7"/>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A127" s="7"/>
+      <c r="B127" s="7"/>
+      <c r="C127" s="7"/>
+      <c r="D127" s="7"/>
+      <c r="E127" s="7"/>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A128" s="7"/>
+      <c r="B128" s="7"/>
+      <c r="C128" s="7"/>
+      <c r="D128" s="7"/>
+      <c r="E128" s="7"/>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A129" s="7"/>
+      <c r="B129" s="7"/>
+      <c r="C129" s="7"/>
+      <c r="D129" s="7"/>
+      <c r="E129" s="7"/>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A130" s="7"/>
+      <c r="B130" s="7"/>
+      <c r="C130" s="7"/>
+      <c r="D130" s="7"/>
+      <c r="E130" s="7"/>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A131" s="7"/>
+      <c r="B131" s="7"/>
+      <c r="C131" s="7"/>
+      <c r="D131" s="7"/>
+      <c r="E131" s="7"/>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A132" s="7"/>
+      <c r="B132" s="7"/>
+      <c r="C132" s="7"/>
+      <c r="D132" s="7"/>
+      <c r="E132" s="7"/>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A133" s="7"/>
+      <c r="B133" s="7"/>
+      <c r="C133" s="7"/>
+      <c r="D133" s="7"/>
+      <c r="E133" s="7"/>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A134" s="7"/>
+      <c r="B134" s="7"/>
+      <c r="C134" s="7"/>
+      <c r="D134" s="7"/>
+      <c r="E134" s="7"/>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A135" s="7"/>
+      <c r="B135" s="7"/>
+      <c r="C135" s="7"/>
+      <c r="D135" s="7"/>
+      <c r="E135" s="7"/>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A136" s="7"/>
+      <c r="B136" s="7"/>
+      <c r="C136" s="7"/>
+      <c r="D136" s="7"/>
+      <c r="E136" s="7"/>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A137" s="7"/>
+      <c r="B137" s="7"/>
+      <c r="C137" s="7"/>
+      <c r="D137" s="7"/>
+      <c r="E137" s="7"/>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A138" s="7"/>
+      <c r="B138" s="7"/>
+      <c r="C138" s="7"/>
+      <c r="D138" s="7"/>
+      <c r="E138" s="7"/>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A139" s="7"/>
+      <c r="B139" s="7"/>
+      <c r="C139" s="7"/>
+      <c r="D139" s="7"/>
+      <c r="E139" s="7"/>
     </row>
   </sheetData>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="E19:E29">
-    <sortCondition ref="E19:E29"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="E16">
+    <sortCondition ref="E16"/>
   </sortState>
+  <mergeCells count="1">
+    <mergeCell ref="A114:E139"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100CA5D0A6329BB324E86983B32928CFC2E" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3d7eac4bce3bbb09c82bd908806be82e">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9e0b35a9-e6cb-436b-81d4-4440ba439ca5" xmlns:ns3="ced60a7f-99b1-48d2-b555-34851c8026ae" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="eb51570e5b7cb8bd524bc2df5324d4a3" ns2:_="" ns3:_="">
     <xsd:import namespace="9e0b35a9-e6cb-436b-81d4-4440ba439ca5"/>
@@ -3238,6 +3617,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3250,14 +3638,6 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D48FB9E6-6DE3-40FB-81F7-677295638F7C}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6414E68-BBC1-4A96-B078-EF7EE95D29CE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3276,6 +3656,14 @@
 </ds:datastoreItem>
 </file>
 
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D48FB9E6-6DE3-40FB-81F7-677295638F7C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1EE6EC55-B0E7-4ACE-A5DA-E03DCA4973DE}">
   <ds:schemaRefs>

</xml_diff>